<commit_message>
Deployed 4ae3c36 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/artifacts/soma.xlsx
+++ b/artifacts/soma.xlsx
@@ -23,42 +23,44 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpirometryProtocol" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MolecularAssayProtocol" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuantityValue" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NamedEntity" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellTypeReference" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpeciesReference" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChemicalEntityReference" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnatomicalEntityReference" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExposureCondition" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellularSystem" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellLine" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellCultureConditions" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellCultureMedium" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MediumSupplement" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuantityRange" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CiliaryFunctionAssay" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CiliaryFunctionOutput" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASLAssay" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASLOutput" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MucociliaryClearanceAssay" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MucociliaryClearanceOutput" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OxidativeStressAssay" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OxidativeStressOutput" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionAssay" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionOutput" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGFRSignalingAssay" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGFRSignalingOutput" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellAssay" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellOutput" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumAssay" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumOutput" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionAssay" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionOutput" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoxJExpressionAssay" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoxJExpressionOutput" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionAssay" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionOutput" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variability" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NamedEntity" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellTypeReference" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpeciesReference" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChemicalEntityReference" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnatomicalEntityReference" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExposureCondition" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResponseComparison" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellularSystem" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellLine" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellCultureConditions" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellCultureMedium" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MediumSupplement" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuantityRange" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CiliaryFunctionAssay" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CiliaryFunctionOutput" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASLAssay" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASLOutput" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MucociliaryClearanceAssay" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MucociliaryClearanceOutput" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OxidativeStressAssay" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OxidativeStressOutput" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionAssay" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionOutput" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGFRSignalingAssay" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGFRSignalingOutput" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellAssay" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellOutput" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumAssay" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumOutput" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionAssay" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionOutput" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoxJExpressionAssay" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoxJExpressionOutput" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionAssay" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionOutput" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container" sheetId="54" state="visible" r:id="rId54"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1121,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1135,8 +1137,28 @@
           <t>unit</t>
         </is>
       </c>
-    </row>
-  </sheetData>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>central_tendency</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>variability</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sample_size</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"mean,median,geometric_mean,single_value"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1147,22 +1169,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>variability_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>lower_bound</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>upper_bound</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"standard_deviation,standard_error,confidence_interval_95,confidence_interval_other,range,interquartile_range"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1387,6 +1429,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1427,7 +1495,99 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>derived_from_assay</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>compared_measurement</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>control_output</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>treated_output</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>change_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>change_direction</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>change_value</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>p_value</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>statistical_test</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>derivation</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"absolute_difference,percent_change,fold_change,ratio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"increased,decreased,no_change"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"reported_in_paper,computed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1571,7 +1731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1637,7 +1797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1706,7 +1866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1769,88 +1929,6 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>name</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>supplement_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>concentration</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>manufacturer</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>catalog_number</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"growth_factor,antibiotic,antifungal,hormone,vitamin,amino_acid,lipid,trace_element,attachment_factor,differentiation_factor"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>min_value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>max_value</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>unit</t>
         </is>
       </c>
     </row>
@@ -1929,6 +2007,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>supplement_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>catalog_number</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"growth_factor,antibiotic,antifungal,hormone,vitamin,amino_acid,lipid,trace_element,attachment_factor,differentiation_factor"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>min_value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>max_value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1994,13 +2154,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2046,31 +2206,44 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>experimental_group</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>measured_under</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"coordinated,dyskinetic,immotile,rotational,stiff"</formula1>
     </dataValidation>
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2131,13 +2304,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H1"/>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2168,26 +2341,41 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>experimental_group</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>measured_under</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2253,13 +2441,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H1"/>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2290,31 +2478,44 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>experimental_group</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>measured_under</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"normal,reversed,absent,variable"</formula1>
     </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2380,13 +2581,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2482,153 +2683,36 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>experimental_group</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>measured_under</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>stimulation_agent</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>inhibitor_used</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>informs_on_key_event</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>study_subject</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>has_exposure_condition</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>follows_protocols</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>has_specified_output</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>assay_date</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>cftr_chloride_secretion</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>cftr_forskolin_response</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>inhibitor_sensitive_current</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cftr_specific_current</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>sweat_chloride_concentration</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>nasal_potential_difference</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2701,6 +2785,153 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>stimulation_agent</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>inhibitor_used</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>informs_on_key_event</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>study_subject</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>has_exposure_condition</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>follows_protocols</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>has_specified_output</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>assay_date</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>cftr_chloride_secretion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>cftr_forskolin_response</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>inhibitor_sensitive_current</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cftr_specific_current</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sweat_chloride_concentration</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>nasal_potential_difference</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>experimental_group</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>measured_under</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>normalization_reference</t>
         </is>
       </c>
@@ -2760,7 +2991,447 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>egfr_phosphorylation_y1068</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>egfr_phosphorylation_y1173</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>total_egfr_protein</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>downstream_kinase_activation</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>erk_phosphorylation</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>akt_phosphorylation</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>pathway_biomarkers</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>egfr_ligand_expression</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>egfr_membrane_localization</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>experimental_group</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>measured_under</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>informs_on_key_event</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>study_subject</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>has_exposure_condition</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>follows_protocols</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>has_specified_output</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>assay_date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>goblet_cell_count</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>goblet_cell_percentage</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>muc5ac_mrna_expression</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>muc5ac_protein_expression</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>muc5b_mrna_expression</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>muc5b_protein_expression</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>muc5ac_muc5b_ratio</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>mucin_protein_concentration</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>mucin_secretion_rate</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>percent_solids</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>goblet_to_ciliated_ratio</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>mucus_viscosity</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>experimental_group</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>measured_under</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>target_cell_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>informs_on_key_event</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>study_subject</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>has_exposure_condition</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>follows_protocols</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>has_specified_output</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>assay_date</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>neutrophil_percentage</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>eosinophil_percentage</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>macrophage_percentage</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>lymphocyte_percentage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>total_cell_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>il6_concentration</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>il8_concentration</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>tnf_alpha_concentration</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>il1_beta_concentration</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>total_protein_concentration</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>alpha_diversity</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>beta_diversity</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>bacterial_load</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>cell_free_dna</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>experimental_group</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>measured_under</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2772,47 +3443,47 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>egfr_phosphorylation_y1068</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>egfr_phosphorylation_y1173</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>total_egfr_protein</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>downstream_kinase_activation</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>erk_phosphorylation</t>
+          <t>reference_dataset</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hemoglobin_level</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>recent_respiratory_illness</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>informs_on_key_event</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>study_subject</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>akt_phosphorylation</t>
+          <t>has_exposure_condition</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>pathway_biomarkers</t>
+          <t>follows_protocols</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>egfr_ligand_expression</t>
+          <t>has_specified_output</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>egfr_membrane_localization</t>
+          <t>assay_date</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -2836,7 +3507,128 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fev1</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fvc</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fev1_fvc_ratio</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>feno</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>decline_rate</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>bronchodilator_response</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dlco</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>peak_expiratory_flow</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>fef25_75</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>total_lung_capacity</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>functional_residual_capacity</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>residual_volume</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>lung_compliance</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>lung_elastance</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>lung_resistance</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>experimental_group</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>measured_under</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2848,6 +3640,67 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>aopwiki_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>molecular_initiating_event</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>key_events</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>key_event_relationships</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>adverse_outcome</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>stressors</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>informs_on_key_event</t>
         </is>
       </c>
@@ -2897,817 +3750,295 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>goblet_cell_count</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>goblet_cell_percentage</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>muc5ac_mrna_expression</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>muc5ac_protein_expression</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>muc5b_mrna_expression</t>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>foxj1_mrna_expression</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>foxj1_protein_expression</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>foxj1_positive_cell_percentage</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>foxj1_nuclear_localization</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>experimental_group</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>muc5b_protein_expression</t>
+          <t>measured_under</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>muc5ac_muc5b_ratio</t>
+          <t>id</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>mucin_protein_concentration</t>
+          <t>name</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>mucin_secretion_rate</t>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>target_gene</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>gene_expression_method</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>normalization_reference</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>informs_on_key_event</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>study_subject</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>has_exposure_condition</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>follows_protocols</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>has_specified_output</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>assay_date</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>percent_solids</t>
+          <t>id</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>goblet_to_ciliated_ratio</t>
+          <t>name</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>mucus_viscosity</t>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>mrna_level</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>protein_level</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>percentage_positive_cells</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>experimental_group</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>measured_under</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"control,vehicle_control,baseline,treated,recovery,sham"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>key_events</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>key_event_relationships</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>adverse_outcome_pathways</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>response_comparisons</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ciliary_function_assays</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>asl_assays</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>mcc_assays</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>oxidative_stress_assays</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>cftr_assays</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>egfr_signaling_assays</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>goblet_cell_assays</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>balf_sputum_assays</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>lung_function_assays</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>foxj_assays</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>target_cell_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>informs_on_key_event</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>study_subject</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>has_exposure_condition</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>follows_protocols</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>has_specified_output</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>assay_date</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>neutrophil_percentage</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>eosinophil_percentage</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>macrophage_percentage</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>lymphocyte_percentage</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>total_cell_count</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>il6_concentration</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>il8_concentration</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>tnf_alpha_concentration</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>il1_beta_concentration</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>total_protein_concentration</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>alpha_diversity</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>beta_diversity</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>bacterial_load</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>cell_free_dna</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>id</t>
+          <t>gene_expression_assays</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>reference_dataset</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>hemoglobin_level</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>recent_respiratory_illness</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>informs_on_key_event</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>study_subject</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>has_exposure_condition</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>follows_protocols</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>has_specified_output</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>assay_date</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>fev1</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>fvc</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>fev1_fvc_ratio</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>feno</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>decline_rate</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>bronchodilator_response</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>dlco</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>peak_expiratory_flow</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>fef25_75</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>total_lung_capacity</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>functional_residual_capacity</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>residual_volume</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>lung_compliance</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>lung_elastance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>lung_resistance</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>informs_on_key_event</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>study_subject</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>has_exposure_condition</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>follows_protocols</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>has_specified_output</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>assay_date</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>foxj1_mrna_expression</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>foxj1_protein_expression</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>foxj1_positive_cell_percentage</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>foxj1_nuclear_localization</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>aopwiki_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>molecular_initiating_event</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>key_events</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>key_event_relationships</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>adverse_outcome</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>stressors</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>target_gene</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>gene_expression_method</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>normalization_reference</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>informs_on_key_event</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>study_subject</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>has_exposure_condition</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>follows_protocols</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>has_specified_output</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>assay_date</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>mrna_level</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>protein_level</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>percentage_positive_cells</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>key_events</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>adverse_outcome_pathways</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ciliary_function_assays</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>asl_assays</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>mcc_assays</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>oxidative_stress_assays</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>cftr_assays</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>egfr_signaling_assays</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>goblet_cell_assays</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>balf_sputum_assays</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>lung_function_assays</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>foxj_assays</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>gene_expression_assays</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
         <is>
           <t>protocols</t>
         </is>

</xml_diff>

<commit_message>
Deployed 4ffffdc with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/artifacts/soma.xlsx
+++ b/artifacts/soma.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -614,25 +614,30 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>member_of_cohort</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>subject_type</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>model_species</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Deployed 70e8d07 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/artifacts/soma.xlsx
+++ b/artifacts/soma.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,14 +502,27 @@
           <t>explanation</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>article_section</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>figure_reference</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SUPPORT,REFUTE,NO_EVIDENCE"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"HUMAN_CLINICAL,MODEL_ORGANISM,IN_VITRO,COMPUTATIONAL,OTHER"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"abstract,introduction,methods,results,discussion,figure_caption,table,supplementary"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2241,7 +2254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2302,15 +2315,20 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2401,7 +2419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2447,15 +2465,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2548,7 +2571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2594,15 +2617,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2787,7 +2815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2898,15 +2926,20 @@
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3004,7 +3037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3055,15 +3088,20 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3161,7 +3199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3227,15 +3265,20 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3323,7 +3366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3404,15 +3447,20 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3505,7 +3553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3596,15 +3644,20 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3776,7 +3829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3872,15 +3925,20 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3968,7 +4026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4009,15 +4067,20 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -4120,7 +4183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4156,15 +4219,20 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data_in_figure_only</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>